<commit_message>
Lên version 1.2.2: bổ sung thông tin tổng số tín chỉ trong quản lý phân loại kết quả học tập, rèn luyện.
</commit_message>
<xml_diff>
--- a/media/com_eqa/xlsx/sample_conduct_performance.xlsx
+++ b/media/com_eqa/xlsx/sample_conduct_performance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Temporary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFF47DE9-0B5D-4E50-BBF4-398549CB3EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5261515D-6AC5-407C-8712-A7CA5701F66D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{ADDE22B4-7847-444B-95F7-E223B0D12C89}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="129">
   <si>
     <t>TT</t>
   </si>
@@ -418,6 +418,9 @@
   </si>
   <si>
     <t>TEST- KẾT QUẢ PHÂN LOẠI HỌC VIÊN LỚP</t>
+  </si>
+  <si>
+    <t>Số TC</t>
   </si>
 </sst>
 </file>
@@ -587,7 +590,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -662,11 +665,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -799,47 +813,68 @@
     <xf numFmtId="49" fontId="22" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1189,7 +1224,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O59"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.08984375" customWidth="1"/>
@@ -1202,52 +1237,55 @@
     <col min="8" max="8" width="3.08984375" customWidth="1"/>
     <col min="9" max="9" width="3.36328125" customWidth="1"/>
     <col min="10" max="10" width="3.453125" customWidth="1"/>
-    <col min="11" max="11" width="7.54296875" customWidth="1"/>
-    <col min="12" max="12" width="6" customWidth="1"/>
-    <col min="13" max="13" width="5.54296875" customWidth="1"/>
-    <col min="14" max="14" width="6" customWidth="1"/>
-    <col min="15" max="15" width="7" customWidth="1"/>
+    <col min="11" max="11" width="5.81640625" customWidth="1"/>
+    <col min="12" max="12" width="7.54296875" customWidth="1"/>
+    <col min="13" max="13" width="6" customWidth="1"/>
+    <col min="14" max="14" width="5.54296875" customWidth="1"/>
+    <col min="15" max="15" width="6" customWidth="1"/>
+    <col min="16" max="16" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:16" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="61" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="48"/>
-    </row>
-    <row r="2" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="A2" s="49" t="s">
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="61"/>
+    </row>
+    <row r="2" spans="1:16" ht="18" x14ac:dyDescent="0.35">
+      <c r="A2" s="62" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="49"/>
-    </row>
-    <row r="3" spans="1:15" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+    </row>
+    <row r="3" spans="1:16" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1263,95 +1301,101 @@
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
-    </row>
-    <row r="4" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="50" t="s">
+      <c r="P3" s="1"/>
+    </row>
+    <row r="4" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="51" t="s">
+      <c r="B4" s="63" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="50" t="s">
+      <c r="C4" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="50" t="s">
+      <c r="D4" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="52" t="s">
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="52" t="s">
+      <c r="H4" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="52" t="s">
+      <c r="I4" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="52" t="s">
+      <c r="J4" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="53" t="s">
+      <c r="K4" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="L4" s="53"/>
-      <c r="M4" s="50" t="s">
+      <c r="L4" s="67"/>
+      <c r="M4" s="68"/>
+      <c r="N4" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="50"/>
-      <c r="O4" s="50" t="s">
+      <c r="O4" s="58"/>
+      <c r="P4" s="58" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="12.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="50"/>
-      <c r="B5" s="54"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="53" t="s">
+    <row r="5" spans="1:16" ht="12.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="58"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="53" t="s">
+      <c r="E5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="53" t="s">
+      <c r="F5" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="2" t="s">
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="48" t="s">
+        <v>128</v>
+      </c>
+      <c r="L5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="M5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M5" s="52" t="s">
+      <c r="N5" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="N5" s="52" t="s">
+      <c r="O5" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="O5" s="50"/>
-    </row>
-    <row r="6" spans="1:15" ht="13.65" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="51"/>
+      <c r="P5" s="58"/>
+    </row>
+    <row r="6" spans="1:16" ht="13.65" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="63"/>
       <c r="B6" s="45"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="52"/>
-      <c r="N6" s="52"/>
-      <c r="O6" s="50"/>
-    </row>
-    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C6" s="63"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="60"/>
+      <c r="H6" s="60"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="60"/>
+      <c r="K6" s="65"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="60"/>
+      <c r="O6" s="60"/>
+      <c r="P6" s="58"/>
+    </row>
+    <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6">
         <v>1</v>
       </c>
@@ -1372,23 +1416,26 @@
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
       <c r="J7" s="4"/>
-      <c r="K7" s="8">
+      <c r="K7" s="4">
+        <v>17</v>
+      </c>
+      <c r="L7" s="8">
         <v>2.82</v>
       </c>
-      <c r="L7" s="9" t="s">
+      <c r="M7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M7" s="6">
+      <c r="N7" s="6">
         <v>89</v>
       </c>
-      <c r="N7" s="10" t="s">
+      <c r="O7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="11" t="s">
+      <c r="P7" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6">
         <v>2</v>
       </c>
@@ -1405,21 +1452,24 @@
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
       <c r="J8" s="4"/>
-      <c r="K8" s="8">
+      <c r="K8" s="4">
+        <v>19</v>
+      </c>
+      <c r="L8" s="8">
         <v>2.15</v>
       </c>
-      <c r="L8" s="40" t="s">
+      <c r="M8" s="40" t="s">
         <v>68</v>
       </c>
-      <c r="M8" s="6">
+      <c r="N8" s="6">
         <v>84</v>
       </c>
-      <c r="N8" s="10" t="s">
+      <c r="O8" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="12"/>
-    </row>
-    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P8" s="12"/>
+    </row>
+    <row r="9" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6">
         <v>3</v>
       </c>
@@ -1438,21 +1488,24 @@
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="4"/>
-      <c r="K9" s="8">
+      <c r="K9" s="4">
+        <v>17</v>
+      </c>
+      <c r="L9" s="8">
         <v>2.2400000000000002</v>
       </c>
-      <c r="L9" s="40" t="s">
+      <c r="M9" s="40" t="s">
         <v>68</v>
       </c>
-      <c r="M9" s="6">
+      <c r="N9" s="6">
         <v>85</v>
       </c>
-      <c r="N9" s="10" t="s">
+      <c r="O9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="11"/>
-    </row>
-    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P9" s="11"/>
+    </row>
+    <row r="10" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
         <v>4</v>
       </c>
@@ -1469,21 +1522,24 @@
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
       <c r="J10" s="4"/>
-      <c r="K10" s="8">
+      <c r="K10" s="4">
+        <v>17</v>
+      </c>
+      <c r="L10" s="8">
         <v>2.41</v>
       </c>
-      <c r="L10" s="35" t="s">
+      <c r="M10" s="35" t="s">
         <v>68</v>
       </c>
-      <c r="M10" s="6">
+      <c r="N10" s="6">
         <v>85</v>
       </c>
-      <c r="N10" s="10" t="s">
+      <c r="O10" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="14"/>
-    </row>
-    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P10" s="14"/>
+    </row>
+    <row r="11" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6">
         <v>5</v>
       </c>
@@ -1504,23 +1560,26 @@
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="4"/>
-      <c r="K11" s="8">
+      <c r="K11" s="4">
+        <v>17</v>
+      </c>
+      <c r="L11" s="8">
         <v>3.24</v>
       </c>
-      <c r="L11" s="9" t="s">
+      <c r="M11" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="M11" s="6">
+      <c r="N11" s="6">
         <v>90</v>
       </c>
-      <c r="N11" s="10" t="s">
+      <c r="O11" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="O11" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P11" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6">
         <v>6</v>
       </c>
@@ -1537,21 +1596,24 @@
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="4"/>
-      <c r="K12" s="8">
+      <c r="K12" s="4">
+        <v>17</v>
+      </c>
+      <c r="L12" s="8">
         <v>2.91</v>
       </c>
-      <c r="L12" s="9" t="s">
+      <c r="M12" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M12" s="6">
+      <c r="N12" s="6">
         <v>87</v>
       </c>
-      <c r="N12" s="10" t="s">
+      <c r="O12" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O12" s="11"/>
-    </row>
-    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P12" s="11"/>
+    </row>
+    <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6">
         <v>7</v>
       </c>
@@ -1568,21 +1630,24 @@
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
       <c r="J13" s="4"/>
-      <c r="K13" s="8">
+      <c r="K13" s="4">
+        <v>17</v>
+      </c>
+      <c r="L13" s="8">
         <v>2.68</v>
       </c>
-      <c r="L13" s="9" t="s">
+      <c r="M13" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M13" s="6">
+      <c r="N13" s="6">
         <v>85</v>
       </c>
-      <c r="N13" s="10" t="s">
+      <c r="O13" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O13" s="12"/>
-    </row>
-    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P13" s="12"/>
+    </row>
+    <row r="14" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="6">
         <v>8</v>
       </c>
@@ -1603,21 +1668,24 @@
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="4"/>
-      <c r="K14" s="8">
+      <c r="K14" s="4">
+        <v>17</v>
+      </c>
+      <c r="L14" s="8">
         <v>2.5</v>
       </c>
-      <c r="L14" s="9" t="s">
+      <c r="M14" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M14" s="6">
+      <c r="N14" s="6">
         <v>85</v>
       </c>
-      <c r="N14" s="10" t="s">
+      <c r="O14" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O14" s="39"/>
-    </row>
-    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P14" s="39"/>
+    </row>
+    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6">
         <v>9</v>
       </c>
@@ -1638,21 +1706,24 @@
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
       <c r="J15" s="4"/>
-      <c r="K15" s="8">
+      <c r="K15" s="4">
+        <v>17</v>
+      </c>
+      <c r="L15" s="8">
         <v>2.38</v>
       </c>
-      <c r="L15" s="9" t="s">
+      <c r="M15" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M15" s="6">
+      <c r="N15" s="6">
         <v>84</v>
       </c>
-      <c r="N15" s="10" t="s">
+      <c r="O15" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O15" s="13"/>
-    </row>
-    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P15" s="13"/>
+    </row>
+    <row r="16" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6">
         <v>10</v>
       </c>
@@ -1669,21 +1740,24 @@
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
       <c r="J16" s="4"/>
-      <c r="K16" s="8">
+      <c r="K16" s="4">
+        <v>17</v>
+      </c>
+      <c r="L16" s="8">
         <v>2.3199999999999998</v>
       </c>
-      <c r="L16" s="9" t="s">
+      <c r="M16" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M16" s="6">
+      <c r="N16" s="6">
         <v>84</v>
       </c>
-      <c r="N16" s="10" t="s">
+      <c r="O16" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O16" s="13"/>
-    </row>
-    <row r="17" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P16" s="13"/>
+    </row>
+    <row r="17" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6">
         <v>11</v>
       </c>
@@ -1702,21 +1776,24 @@
       </c>
       <c r="I17" s="6"/>
       <c r="J17" s="4"/>
-      <c r="K17" s="8">
+      <c r="K17" s="4">
+        <v>17</v>
+      </c>
+      <c r="L17" s="8">
         <v>2.2400000000000002</v>
       </c>
-      <c r="L17" s="9" t="s">
+      <c r="M17" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M17" s="6">
+      <c r="N17" s="6">
         <v>84</v>
       </c>
-      <c r="N17" s="10" t="s">
+      <c r="O17" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O17" s="14"/>
-    </row>
-    <row r="18" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P17" s="14"/>
+    </row>
+    <row r="18" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6">
         <v>12</v>
       </c>
@@ -1733,21 +1810,24 @@
       <c r="H18" s="6"/>
       <c r="I18" s="6"/>
       <c r="J18" s="4"/>
-      <c r="K18" s="8">
+      <c r="K18" s="4">
+        <v>19</v>
+      </c>
+      <c r="L18" s="8">
         <v>2.2400000000000002</v>
       </c>
-      <c r="L18" s="9" t="s">
+      <c r="M18" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M18" s="6">
+      <c r="N18" s="6">
         <v>84</v>
       </c>
-      <c r="N18" s="10" t="s">
+      <c r="O18" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O18" s="11"/>
-    </row>
-    <row r="19" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P18" s="11"/>
+    </row>
+    <row r="19" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6">
         <v>13</v>
       </c>
@@ -1770,21 +1850,24 @@
       </c>
       <c r="I19" s="6"/>
       <c r="J19" s="4"/>
-      <c r="K19" s="8">
+      <c r="K19" s="4">
+        <v>17</v>
+      </c>
+      <c r="L19" s="8">
         <v>2.38</v>
       </c>
-      <c r="L19" s="9" t="s">
+      <c r="M19" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M19" s="6">
+      <c r="N19" s="6">
         <v>84</v>
       </c>
-      <c r="N19" s="10" t="s">
+      <c r="O19" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O19" s="11"/>
-    </row>
-    <row r="20" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P19" s="11"/>
+    </row>
+    <row r="20" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6">
         <v>14</v>
       </c>
@@ -1801,23 +1884,26 @@
       <c r="H20" s="6"/>
       <c r="I20" s="6"/>
       <c r="J20" s="4"/>
-      <c r="K20" s="8">
+      <c r="K20" s="4">
+        <v>17</v>
+      </c>
+      <c r="L20" s="8">
         <v>3.01</v>
       </c>
-      <c r="L20" s="9" t="s">
+      <c r="M20" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M20" s="6">
+      <c r="N20" s="6">
         <v>87</v>
       </c>
-      <c r="N20" s="10" t="s">
+      <c r="O20" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O20" s="11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P20" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6">
         <v>15</v>
       </c>
@@ -1838,21 +1924,24 @@
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
       <c r="J21" s="4"/>
-      <c r="K21" s="8">
+      <c r="K21" s="4">
+        <v>17</v>
+      </c>
+      <c r="L21" s="8">
         <v>2.12</v>
       </c>
-      <c r="L21" s="9" t="s">
+      <c r="M21" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M21" s="6">
+      <c r="N21" s="6">
         <v>83</v>
       </c>
-      <c r="N21" s="10" t="s">
+      <c r="O21" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O21" s="11"/>
-    </row>
-    <row r="22" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P21" s="11"/>
+    </row>
+    <row r="22" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6">
         <v>16</v>
       </c>
@@ -1869,21 +1958,24 @@
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
       <c r="J22" s="4"/>
-      <c r="K22" s="8">
+      <c r="K22" s="4">
+        <v>17</v>
+      </c>
+      <c r="L22" s="8">
         <v>2.54</v>
       </c>
-      <c r="L22" s="9" t="s">
+      <c r="M22" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M22" s="6">
+      <c r="N22" s="6">
         <v>85</v>
       </c>
-      <c r="N22" s="10" t="s">
+      <c r="O22" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O22" s="11"/>
-    </row>
-    <row r="23" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P22" s="11"/>
+    </row>
+    <row r="23" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="6">
         <v>17</v>
       </c>
@@ -1902,21 +1994,24 @@
       </c>
       <c r="I23" s="6"/>
       <c r="J23" s="4"/>
-      <c r="K23" s="8">
+      <c r="K23" s="4">
+        <v>17</v>
+      </c>
+      <c r="L23" s="8">
         <v>2.62</v>
       </c>
-      <c r="L23" s="9" t="s">
+      <c r="M23" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M23" s="6">
+      <c r="N23" s="6">
         <v>85</v>
       </c>
-      <c r="N23" s="10" t="s">
+      <c r="O23" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O23" s="11"/>
-    </row>
-    <row r="24" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P23" s="11"/>
+    </row>
+    <row r="24" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="6">
         <v>18</v>
       </c>
@@ -1933,21 +2028,24 @@
       <c r="H24" s="6"/>
       <c r="I24" s="6"/>
       <c r="J24" s="4"/>
-      <c r="K24" s="8">
+      <c r="K24" s="4">
+        <v>17</v>
+      </c>
+      <c r="L24" s="8">
         <v>3.15</v>
       </c>
-      <c r="L24" s="9" t="s">
+      <c r="M24" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M24" s="6">
+      <c r="N24" s="6">
         <v>88</v>
       </c>
-      <c r="N24" s="10" t="s">
+      <c r="O24" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O24" s="11"/>
-    </row>
-    <row r="25" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P24" s="11"/>
+    </row>
+    <row r="25" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6">
         <v>19</v>
       </c>
@@ -1968,21 +2066,24 @@
       <c r="H25" s="6"/>
       <c r="I25" s="6"/>
       <c r="J25" s="4"/>
-      <c r="K25" s="8">
+      <c r="K25" s="4">
+        <v>17</v>
+      </c>
+      <c r="L25" s="8">
         <v>2.44</v>
       </c>
-      <c r="L25" s="9" t="s">
+      <c r="M25" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M25" s="6">
+      <c r="N25" s="6">
         <v>84</v>
       </c>
-      <c r="N25" s="10" t="s">
+      <c r="O25" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O25" s="13"/>
-    </row>
-    <row r="26" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P25" s="13"/>
+    </row>
+    <row r="26" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="6">
         <v>20</v>
       </c>
@@ -1999,21 +2100,24 @@
       <c r="H26" s="6"/>
       <c r="I26" s="6"/>
       <c r="J26" s="4"/>
-      <c r="K26" s="8">
+      <c r="K26" s="4">
+        <v>17</v>
+      </c>
+      <c r="L26" s="8">
         <v>2.68</v>
       </c>
-      <c r="L26" s="9" t="s">
+      <c r="M26" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M26" s="6">
+      <c r="N26" s="6">
         <v>86</v>
       </c>
-      <c r="N26" s="10" t="s">
+      <c r="O26" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O26" s="11"/>
-    </row>
-    <row r="27" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P26" s="11"/>
+    </row>
+    <row r="27" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="6">
         <v>21</v>
       </c>
@@ -2032,21 +2136,24 @@
       </c>
       <c r="I27" s="6"/>
       <c r="J27" s="4"/>
-      <c r="K27" s="8">
+      <c r="K27" s="4">
+        <v>17</v>
+      </c>
+      <c r="L27" s="8">
         <v>2.56</v>
       </c>
-      <c r="L27" s="9" t="s">
+      <c r="M27" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M27" s="6">
+      <c r="N27" s="6">
         <v>85</v>
       </c>
-      <c r="N27" s="10" t="s">
+      <c r="O27" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O27" s="13"/>
-    </row>
-    <row r="28" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P27" s="13"/>
+    </row>
+    <row r="28" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="6">
         <v>22</v>
       </c>
@@ -2065,21 +2172,24 @@
       </c>
       <c r="I28" s="6"/>
       <c r="J28" s="4"/>
-      <c r="K28" s="8">
+      <c r="K28" s="4">
+        <v>17</v>
+      </c>
+      <c r="L28" s="8">
         <v>2.09</v>
       </c>
-      <c r="L28" s="9" t="s">
+      <c r="M28" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M28" s="6">
+      <c r="N28" s="6">
         <v>82</v>
       </c>
-      <c r="N28" s="10" t="s">
+      <c r="O28" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O28" s="11"/>
-    </row>
-    <row r="29" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P28" s="11"/>
+    </row>
+    <row r="29" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="6">
         <v>23</v>
       </c>
@@ -2096,21 +2206,24 @@
       <c r="H29" s="6"/>
       <c r="I29" s="6"/>
       <c r="J29" s="4"/>
-      <c r="K29" s="8">
+      <c r="K29" s="4">
+        <v>17</v>
+      </c>
+      <c r="L29" s="8">
         <v>2.4500000000000002</v>
       </c>
-      <c r="L29" s="9" t="s">
+      <c r="M29" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M29" s="6">
+      <c r="N29" s="6">
         <v>84</v>
       </c>
-      <c r="N29" s="10" t="s">
+      <c r="O29" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O29" s="11"/>
-    </row>
-    <row r="30" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="P29" s="11"/>
+    </row>
+    <row r="30" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="6">
         <v>24</v>
       </c>
@@ -2129,21 +2242,24 @@
       </c>
       <c r="I30" s="6"/>
       <c r="J30" s="4"/>
-      <c r="K30" s="8">
+      <c r="K30" s="4">
+        <v>19</v>
+      </c>
+      <c r="L30" s="8">
         <v>0.85</v>
       </c>
-      <c r="L30" s="9" t="s">
+      <c r="M30" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="M30" s="6">
+      <c r="N30" s="6">
         <v>75</v>
       </c>
-      <c r="N30" s="10" t="s">
+      <c r="O30" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="O30" s="11"/>
-    </row>
-    <row r="31" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P30" s="11"/>
+    </row>
+    <row r="31" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="6">
         <v>25</v>
       </c>
@@ -2162,21 +2278,24 @@
       </c>
       <c r="I31" s="6"/>
       <c r="J31" s="4"/>
-      <c r="K31" s="8">
+      <c r="K31" s="4">
+        <v>17</v>
+      </c>
+      <c r="L31" s="8">
         <v>1.32</v>
       </c>
-      <c r="L31" s="9" t="s">
+      <c r="M31" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="M31" s="6">
+      <c r="N31" s="6">
         <v>78</v>
       </c>
-      <c r="N31" s="10" t="s">
+      <c r="O31" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="O31" s="11"/>
-    </row>
-    <row r="32" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P31" s="11"/>
+    </row>
+    <row r="32" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="6">
         <v>26</v>
       </c>
@@ -2195,21 +2314,24 @@
       </c>
       <c r="I32" s="6"/>
       <c r="J32" s="4"/>
-      <c r="K32" s="8">
+      <c r="K32" s="4">
+        <v>17</v>
+      </c>
+      <c r="L32" s="8">
         <v>1.5</v>
       </c>
-      <c r="L32" s="9" t="s">
+      <c r="M32" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="M32" s="6">
+      <c r="N32" s="6">
         <v>78</v>
       </c>
-      <c r="N32" s="10" t="s">
+      <c r="O32" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="O32" s="11"/>
-    </row>
-    <row r="33" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P32" s="11"/>
+    </row>
+    <row r="33" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6">
         <v>27</v>
       </c>
@@ -2228,21 +2350,24 @@
       </c>
       <c r="I33" s="6"/>
       <c r="J33" s="4"/>
-      <c r="K33" s="8">
+      <c r="K33" s="4">
+        <v>17</v>
+      </c>
+      <c r="L33" s="8">
         <v>1.1200000000000001</v>
       </c>
-      <c r="L33" s="9" t="s">
+      <c r="M33" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="M33" s="6">
+      <c r="N33" s="6">
         <v>78</v>
       </c>
-      <c r="N33" s="10" t="s">
+      <c r="O33" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="O33" s="11"/>
-    </row>
-    <row r="34" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P33" s="11"/>
+    </row>
+    <row r="34" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="6">
         <v>28</v>
       </c>
@@ -2259,21 +2384,24 @@
       <c r="H34" s="37"/>
       <c r="I34" s="37"/>
       <c r="J34" s="41"/>
-      <c r="K34" s="38">
+      <c r="K34" s="4">
+        <v>17</v>
+      </c>
+      <c r="L34" s="38">
         <v>1.83</v>
       </c>
-      <c r="L34" s="42" t="s">
+      <c r="M34" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="M34" s="37">
+      <c r="N34" s="37">
         <v>78</v>
       </c>
-      <c r="N34" s="43" t="s">
+      <c r="O34" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="O34" s="44"/>
-    </row>
-    <row r="35" spans="1:15" s="17" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P34" s="44"/>
+    </row>
+    <row r="35" spans="1:16" s="17" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="15">
         <v>29</v>
       </c>
@@ -2290,21 +2418,24 @@
       <c r="H35" s="37"/>
       <c r="I35" s="37"/>
       <c r="J35" s="41"/>
-      <c r="K35" s="38">
+      <c r="K35" s="4">
+        <v>17</v>
+      </c>
+      <c r="L35" s="38">
         <v>2.2999999999999998</v>
       </c>
-      <c r="L35" s="42" t="s">
+      <c r="M35" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="M35" s="37">
+      <c r="N35" s="37">
         <v>83</v>
       </c>
-      <c r="N35" s="43" t="s">
+      <c r="O35" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="O35" s="44"/>
-    </row>
-    <row r="36" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P35" s="44"/>
+    </row>
+    <row r="36" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="6">
         <v>30</v>
       </c>
@@ -2323,21 +2454,24 @@
       </c>
       <c r="I36" s="37"/>
       <c r="J36" s="41"/>
-      <c r="K36" s="38">
+      <c r="K36" s="4">
+        <v>17</v>
+      </c>
+      <c r="L36" s="38">
         <v>1.6</v>
       </c>
-      <c r="L36" s="42" t="s">
+      <c r="M36" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="M36" s="37">
+      <c r="N36" s="37">
         <v>77</v>
       </c>
-      <c r="N36" s="43" t="s">
+      <c r="O36" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="O36" s="44"/>
-    </row>
-    <row r="37" spans="1:15" s="17" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P36" s="44"/>
+    </row>
+    <row r="37" spans="1:16" s="17" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="15">
         <v>31</v>
       </c>
@@ -2356,21 +2490,24 @@
       </c>
       <c r="I37" s="37"/>
       <c r="J37" s="41"/>
-      <c r="K37" s="38">
+      <c r="K37" s="4">
+        <v>17</v>
+      </c>
+      <c r="L37" s="38">
         <v>1.97</v>
       </c>
-      <c r="L37" s="42" t="s">
+      <c r="M37" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="M37" s="37">
+      <c r="N37" s="37">
         <v>78</v>
       </c>
-      <c r="N37" s="43" t="s">
+      <c r="O37" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="O37" s="44"/>
-    </row>
-    <row r="38" spans="1:15" s="17" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P37" s="44"/>
+    </row>
+    <row r="38" spans="1:16" s="17" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="15">
         <v>32</v>
       </c>
@@ -2387,21 +2524,24 @@
       <c r="H38" s="37"/>
       <c r="I38" s="37"/>
       <c r="J38" s="41"/>
-      <c r="K38" s="38">
+      <c r="K38" s="4">
+        <v>17</v>
+      </c>
+      <c r="L38" s="38">
         <v>2.2799999999999998</v>
       </c>
-      <c r="L38" s="42" t="s">
+      <c r="M38" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="M38" s="37">
+      <c r="N38" s="37">
         <v>82</v>
       </c>
-      <c r="N38" s="43" t="s">
+      <c r="O38" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="O38" s="44"/>
-    </row>
-    <row r="39" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P38" s="44"/>
+    </row>
+    <row r="39" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="6">
         <v>33</v>
       </c>
@@ -2418,21 +2558,24 @@
       <c r="H39" s="37"/>
       <c r="I39" s="37"/>
       <c r="J39" s="41"/>
-      <c r="K39" s="38">
+      <c r="K39" s="4">
+        <v>17</v>
+      </c>
+      <c r="L39" s="38">
         <v>1.97</v>
       </c>
-      <c r="L39" s="42" t="s">
+      <c r="M39" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="M39" s="37">
+      <c r="N39" s="37">
         <v>79</v>
       </c>
-      <c r="N39" s="43" t="s">
+      <c r="O39" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="O39" s="44"/>
-    </row>
-    <row r="40" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P39" s="44"/>
+    </row>
+    <row r="40" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="6">
         <v>34</v>
       </c>
@@ -2449,21 +2592,24 @@
       <c r="H40" s="37"/>
       <c r="I40" s="37"/>
       <c r="J40" s="41"/>
-      <c r="K40" s="38">
+      <c r="K40" s="4">
+        <v>17</v>
+      </c>
+      <c r="L40" s="38">
         <v>2.2799999999999998</v>
       </c>
-      <c r="L40" s="42" t="s">
+      <c r="M40" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="M40" s="37">
+      <c r="N40" s="37">
         <v>83</v>
       </c>
-      <c r="N40" s="43" t="s">
+      <c r="O40" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="O40" s="44"/>
-    </row>
-    <row r="41" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P40" s="44"/>
+    </row>
+    <row r="41" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="6">
         <v>35</v>
       </c>
@@ -2480,21 +2626,24 @@
       <c r="H41" s="37"/>
       <c r="I41" s="37"/>
       <c r="J41" s="41"/>
-      <c r="K41" s="38">
+      <c r="K41" s="4">
+        <v>17</v>
+      </c>
+      <c r="L41" s="38">
         <v>2.61</v>
       </c>
-      <c r="L41" s="42" t="s">
+      <c r="M41" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="M41" s="37">
+      <c r="N41" s="37">
         <v>85</v>
       </c>
-      <c r="N41" s="43" t="s">
+      <c r="O41" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="O41" s="44"/>
-    </row>
-    <row r="42" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P41" s="44"/>
+    </row>
+    <row r="42" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6">
         <v>36</v>
       </c>
@@ -2511,26 +2660,29 @@
       <c r="H42" s="37"/>
       <c r="I42" s="37"/>
       <c r="J42" s="41"/>
-      <c r="K42" s="38">
+      <c r="K42" s="4">
+        <v>17</v>
+      </c>
+      <c r="L42" s="38">
         <v>2.48</v>
       </c>
-      <c r="L42" s="42" t="s">
+      <c r="M42" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="M42" s="37">
+      <c r="N42" s="37">
         <v>84</v>
       </c>
-      <c r="N42" s="43" t="s">
+      <c r="O42" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="O42" s="44"/>
-    </row>
-    <row r="43" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="56" t="s">
+      <c r="P42" s="44"/>
+    </row>
+    <row r="43" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="B43" s="56"/>
-      <c r="C43" s="56"/>
+      <c r="B43" s="54"/>
+      <c r="C43" s="54"/>
       <c r="D43" s="31">
         <v>45</v>
       </c>
@@ -2545,48 +2697,51 @@
       <c r="I43" s="19"/>
       <c r="J43" s="19"/>
       <c r="K43" s="19"/>
-      <c r="L43" s="20"/>
+      <c r="L43" s="19"/>
       <c r="M43" s="20"/>
       <c r="N43" s="20"/>
-      <c r="O43" s="21"/>
-    </row>
-    <row r="44" spans="1:15" ht="13.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="57" t="s">
+      <c r="O43" s="20"/>
+      <c r="P43" s="21"/>
+    </row>
+    <row r="44" spans="1:16" ht="13.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="B44" s="57"/>
-      <c r="C44" s="57"/>
-      <c r="D44" s="57"/>
-      <c r="E44" s="57"/>
-      <c r="F44" s="57"/>
-      <c r="G44" s="57"/>
-      <c r="H44" s="57"/>
-      <c r="I44" s="57"/>
-      <c r="J44" s="57"/>
-      <c r="K44" s="57"/>
-      <c r="L44" s="57"/>
-      <c r="M44" s="57"/>
-      <c r="N44" s="57"/>
-      <c r="O44" s="57"/>
-    </row>
-    <row r="45" spans="1:15" ht="13.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="57"/>
-      <c r="B45" s="57"/>
-      <c r="C45" s="57"/>
-      <c r="D45" s="57"/>
-      <c r="E45" s="57"/>
-      <c r="F45" s="57"/>
-      <c r="G45" s="57"/>
-      <c r="H45" s="57"/>
-      <c r="I45" s="57"/>
-      <c r="J45" s="57"/>
-      <c r="K45" s="57"/>
-      <c r="L45" s="57"/>
-      <c r="M45" s="57"/>
-      <c r="N45" s="57"/>
-      <c r="O45" s="57"/>
-    </row>
-    <row r="46" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="B44" s="55"/>
+      <c r="C44" s="55"/>
+      <c r="D44" s="55"/>
+      <c r="E44" s="55"/>
+      <c r="F44" s="55"/>
+      <c r="G44" s="55"/>
+      <c r="H44" s="55"/>
+      <c r="I44" s="55"/>
+      <c r="J44" s="55"/>
+      <c r="K44" s="55"/>
+      <c r="L44" s="55"/>
+      <c r="M44" s="55"/>
+      <c r="N44" s="55"/>
+      <c r="O44" s="55"/>
+      <c r="P44" s="55"/>
+    </row>
+    <row r="45" spans="1:16" ht="13.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="55"/>
+      <c r="B45" s="55"/>
+      <c r="C45" s="55"/>
+      <c r="D45" s="55"/>
+      <c r="E45" s="55"/>
+      <c r="F45" s="55"/>
+      <c r="G45" s="55"/>
+      <c r="H45" s="55"/>
+      <c r="I45" s="55"/>
+      <c r="J45" s="55"/>
+      <c r="K45" s="55"/>
+      <c r="L45" s="55"/>
+      <c r="M45" s="55"/>
+      <c r="N45" s="55"/>
+      <c r="O45" s="55"/>
+      <c r="P45" s="55"/>
+    </row>
+    <row r="46" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A46" s="23" t="s">
         <v>21</v>
       </c>
@@ -2605,9 +2760,10 @@
       <c r="L46" s="25"/>
       <c r="M46" s="25"/>
       <c r="N46" s="25"/>
-      <c r="O46" s="26"/>
-    </row>
-    <row r="47" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="O46" s="25"/>
+      <c r="P46" s="26"/>
+    </row>
+    <row r="47" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A47" s="25"/>
       <c r="B47" s="25"/>
       <c r="C47" s="25" t="s">
@@ -2615,22 +2771,23 @@
       </c>
       <c r="D47" s="25"/>
       <c r="E47" s="25"/>
-      <c r="F47" s="58" t="s">
+      <c r="F47" s="51" t="s">
         <v>75</v>
       </c>
-      <c r="G47" s="58"/>
-      <c r="H47" s="58"/>
-      <c r="I47" s="58"/>
-      <c r="J47" s="58"/>
-      <c r="K47" s="25"/>
-      <c r="L47" s="58" t="s">
+      <c r="G47" s="51"/>
+      <c r="H47" s="51"/>
+      <c r="I47" s="51"/>
+      <c r="J47" s="51"/>
+      <c r="K47" s="26"/>
+      <c r="L47" s="25"/>
+      <c r="M47" s="51" t="s">
         <v>76</v>
       </c>
-      <c r="M47" s="58"/>
-      <c r="N47" s="58"/>
-      <c r="O47" s="26"/>
-    </row>
-    <row r="48" spans="1:15" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="N47" s="51"/>
+      <c r="O47" s="51"/>
+      <c r="P47" s="26"/>
+    </row>
+    <row r="48" spans="1:16" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A48" s="25"/>
       <c r="B48" s="25"/>
       <c r="C48" s="25" t="s">
@@ -2638,24 +2795,25 @@
       </c>
       <c r="D48" s="25"/>
       <c r="E48" s="25"/>
-      <c r="F48" s="59" t="s">
+      <c r="F48" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="G48" s="59"/>
-      <c r="H48" s="59"/>
-      <c r="I48" s="59"/>
-      <c r="J48" s="59"/>
-      <c r="K48" s="25"/>
-      <c r="L48" s="26" t="s">
+      <c r="G48" s="56"/>
+      <c r="H48" s="56"/>
+      <c r="I48" s="56"/>
+      <c r="J48" s="56"/>
+      <c r="K48" s="49"/>
+      <c r="L48" s="25"/>
+      <c r="M48" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="M48" s="26" t="s">
+      <c r="N48" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="N48" s="26"/>
-      <c r="O48" s="27"/>
-    </row>
-    <row r="49" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="O48" s="26"/>
+      <c r="P48" s="27"/>
+    </row>
+    <row r="49" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A49" s="23" t="s">
         <v>21</v>
       </c>
@@ -2665,18 +2823,19 @@
       </c>
       <c r="D49" s="25"/>
       <c r="E49" s="25"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="55"/>
-      <c r="J49" s="55"/>
-      <c r="K49" s="25"/>
-      <c r="L49" s="27"/>
+      <c r="F49" s="57"/>
+      <c r="G49" s="57"/>
+      <c r="H49" s="57"/>
+      <c r="I49" s="57"/>
+      <c r="J49" s="57"/>
+      <c r="K49" s="27"/>
+      <c r="L49" s="25"/>
       <c r="M49" s="27"/>
       <c r="N49" s="27"/>
-      <c r="O49" s="26"/>
-    </row>
-    <row r="50" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="O49" s="27"/>
+      <c r="P49" s="26"/>
+    </row>
+    <row r="50" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A50" s="25"/>
       <c r="B50" s="25"/>
       <c r="C50" s="25" t="s">
@@ -2684,22 +2843,23 @@
       </c>
       <c r="D50" s="25"/>
       <c r="E50" s="25"/>
-      <c r="F50" s="58" t="s">
+      <c r="F50" s="51" t="s">
         <v>81</v>
       </c>
-      <c r="G50" s="58"/>
-      <c r="H50" s="58"/>
-      <c r="I50" s="58"/>
-      <c r="J50" s="58"/>
-      <c r="K50" s="58"/>
-      <c r="L50" s="58" t="s">
+      <c r="G50" s="51"/>
+      <c r="H50" s="51"/>
+      <c r="I50" s="51"/>
+      <c r="J50" s="51"/>
+      <c r="K50" s="51"/>
+      <c r="L50" s="51"/>
+      <c r="M50" s="51" t="s">
         <v>82</v>
       </c>
-      <c r="M50" s="58"/>
-      <c r="N50" s="58"/>
-      <c r="O50" s="26"/>
-    </row>
-    <row r="51" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="N50" s="51"/>
+      <c r="O50" s="51"/>
+      <c r="P50" s="26"/>
+    </row>
+    <row r="51" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A51" s="25"/>
       <c r="B51" s="25"/>
       <c r="C51" s="25" t="s">
@@ -2707,45 +2867,47 @@
       </c>
       <c r="D51" s="25"/>
       <c r="E51" s="25"/>
-      <c r="F51" s="58" t="s">
+      <c r="F51" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="G51" s="58"/>
-      <c r="H51" s="58"/>
-      <c r="I51" s="58"/>
-      <c r="J51" s="58"/>
-      <c r="K51" s="25"/>
-      <c r="L51" s="58" t="s">
+      <c r="G51" s="51"/>
+      <c r="H51" s="51"/>
+      <c r="I51" s="51"/>
+      <c r="J51" s="51"/>
+      <c r="K51" s="26"/>
+      <c r="L51" s="25"/>
+      <c r="M51" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="M51" s="58"/>
-      <c r="N51" s="58"/>
-      <c r="O51" s="58"/>
-    </row>
-    <row r="52" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="N51" s="51"/>
+      <c r="O51" s="51"/>
+      <c r="P51" s="51"/>
+    </row>
+    <row r="52" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A52" s="23" t="s">
         <v>21</v>
       </c>
       <c r="B52" s="23"/>
-      <c r="C52" s="60" t="s">
+      <c r="C52" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="D52" s="60"/>
-      <c r="E52" s="60"/>
-      <c r="F52" s="60"/>
-      <c r="G52" s="60"/>
-      <c r="H52" s="60"/>
-      <c r="I52" s="60"/>
-      <c r="J52" s="60"/>
-      <c r="K52" s="25"/>
-      <c r="L52" s="60" t="s">
+      <c r="D52" s="53"/>
+      <c r="E52" s="53"/>
+      <c r="F52" s="53"/>
+      <c r="G52" s="53"/>
+      <c r="H52" s="53"/>
+      <c r="I52" s="53"/>
+      <c r="J52" s="53"/>
+      <c r="K52" s="50"/>
+      <c r="L52" s="25"/>
+      <c r="M52" s="53" t="s">
         <v>85</v>
       </c>
-      <c r="M52" s="60"/>
-      <c r="N52" s="60"/>
-      <c r="O52" s="60"/>
-    </row>
-    <row r="53" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="N52" s="53"/>
+      <c r="O52" s="53"/>
+      <c r="P52" s="53"/>
+    </row>
+    <row r="53" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A53" s="25"/>
       <c r="B53" s="25"/>
       <c r="C53" s="25" t="s">
@@ -2753,22 +2915,23 @@
       </c>
       <c r="D53" s="25"/>
       <c r="E53" s="25"/>
-      <c r="F53" s="58" t="s">
+      <c r="F53" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="G53" s="58"/>
-      <c r="H53" s="58"/>
-      <c r="I53" s="58"/>
-      <c r="J53" s="58"/>
-      <c r="K53" s="58"/>
-      <c r="L53" s="58" t="s">
+      <c r="G53" s="51"/>
+      <c r="H53" s="51"/>
+      <c r="I53" s="51"/>
+      <c r="J53" s="51"/>
+      <c r="K53" s="51"/>
+      <c r="L53" s="51"/>
+      <c r="M53" s="51" t="s">
         <v>88</v>
       </c>
-      <c r="M53" s="58"/>
-      <c r="N53" s="58"/>
-      <c r="O53" s="58"/>
-    </row>
-    <row r="54" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="N53" s="51"/>
+      <c r="O53" s="51"/>
+      <c r="P53" s="51"/>
+    </row>
+    <row r="54" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A54" s="25"/>
       <c r="B54" s="25"/>
       <c r="C54" s="25" t="s">
@@ -2776,22 +2939,23 @@
       </c>
       <c r="D54" s="25"/>
       <c r="E54" s="25"/>
-      <c r="F54" s="58" t="s">
+      <c r="F54" s="51" t="s">
         <v>89</v>
       </c>
-      <c r="G54" s="58"/>
-      <c r="H54" s="58"/>
-      <c r="I54" s="58"/>
-      <c r="J54" s="58"/>
-      <c r="K54" s="58"/>
-      <c r="L54" s="58" t="s">
+      <c r="G54" s="51"/>
+      <c r="H54" s="51"/>
+      <c r="I54" s="51"/>
+      <c r="J54" s="51"/>
+      <c r="K54" s="51"/>
+      <c r="L54" s="51"/>
+      <c r="M54" s="51" t="s">
         <v>71</v>
       </c>
-      <c r="M54" s="58"/>
-      <c r="N54" s="58"/>
-      <c r="O54" s="58"/>
-    </row>
-    <row r="55" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="N54" s="51"/>
+      <c r="O54" s="51"/>
+      <c r="P54" s="51"/>
+    </row>
+    <row r="55" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A55" s="25"/>
       <c r="B55" s="25"/>
       <c r="C55" s="25"/>
@@ -2806,32 +2970,34 @@
       <c r="L55" s="25"/>
       <c r="M55" s="25"/>
       <c r="N55" s="25"/>
-      <c r="O55" s="22"/>
-    </row>
-    <row r="56" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="O55" s="25"/>
+      <c r="P55" s="22"/>
+    </row>
+    <row r="56" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A56" s="25"/>
       <c r="B56" s="25"/>
       <c r="C56" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="D56" s="61" t="s">
+      <c r="D56" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="E56" s="61"/>
-      <c r="F56" s="61"/>
-      <c r="G56" s="61"/>
-      <c r="H56" s="61"/>
-      <c r="I56" s="61" t="s">
+      <c r="E56" s="52"/>
+      <c r="F56" s="52"/>
+      <c r="G56" s="52"/>
+      <c r="H56" s="52"/>
+      <c r="I56" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="J56" s="61"/>
-      <c r="K56" s="61"/>
-      <c r="L56" s="61"/>
-      <c r="M56" s="61"/>
-      <c r="N56" s="61"/>
-      <c r="O56" s="61"/>
-    </row>
-    <row r="57" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="J56" s="52"/>
+      <c r="K56" s="52"/>
+      <c r="L56" s="52"/>
+      <c r="M56" s="52"/>
+      <c r="N56" s="52"/>
+      <c r="O56" s="52"/>
+      <c r="P56" s="52"/>
+    </row>
+    <row r="57" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A57" s="25"/>
       <c r="B57" s="25"/>
       <c r="C57" s="22"/>
@@ -2847,8 +3013,9 @@
       <c r="M57" s="22"/>
       <c r="N57" s="22"/>
       <c r="O57" s="22"/>
-    </row>
-    <row r="58" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="P57" s="22"/>
+    </row>
+    <row r="58" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A58" s="25"/>
       <c r="B58" s="25"/>
       <c r="C58" s="22"/>
@@ -2864,8 +3031,9 @@
       <c r="M58" s="22"/>
       <c r="N58" s="22"/>
       <c r="O58" s="22"/>
-    </row>
-    <row r="59" spans="1:15" ht="18" x14ac:dyDescent="0.4">
+      <c r="P58" s="22"/>
+    </row>
+    <row r="59" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A59" s="25"/>
       <c r="B59" s="25"/>
       <c r="C59" s="22"/>
@@ -2881,36 +3049,12 @@
       <c r="M59" s="22"/>
       <c r="N59" s="22"/>
       <c r="O59" s="22"/>
+      <c r="P59" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="F53:K53"/>
-    <mergeCell ref="L53:O53"/>
-    <mergeCell ref="F54:K54"/>
-    <mergeCell ref="L54:O54"/>
-    <mergeCell ref="D56:H56"/>
-    <mergeCell ref="I56:O56"/>
-    <mergeCell ref="F50:K50"/>
-    <mergeCell ref="L50:N50"/>
-    <mergeCell ref="F51:J51"/>
-    <mergeCell ref="L51:O51"/>
-    <mergeCell ref="C52:J52"/>
-    <mergeCell ref="L52:O52"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="A44:O45"/>
-    <mergeCell ref="F47:J47"/>
-    <mergeCell ref="L47:N47"/>
-    <mergeCell ref="F48:J48"/>
-    <mergeCell ref="F49:J49"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="O4:O6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="M5:M6"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
     <mergeCell ref="A4:A6"/>
     <mergeCell ref="C4:C6"/>
     <mergeCell ref="D4:F4"/>
@@ -2918,8 +3062,33 @@
     <mergeCell ref="H4:H6"/>
     <mergeCell ref="I4:I6"/>
     <mergeCell ref="J4:J6"/>
-    <mergeCell ref="K4:L4"/>
     <mergeCell ref="B4:B5"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="F49:J49"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="P4:P6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A44:P45"/>
+    <mergeCell ref="F47:J47"/>
+    <mergeCell ref="M47:O47"/>
+    <mergeCell ref="F48:J48"/>
+    <mergeCell ref="F50:L50"/>
+    <mergeCell ref="M50:O50"/>
+    <mergeCell ref="F51:J51"/>
+    <mergeCell ref="M51:P51"/>
+    <mergeCell ref="C52:J52"/>
+    <mergeCell ref="M52:P52"/>
+    <mergeCell ref="F53:L53"/>
+    <mergeCell ref="M53:P53"/>
+    <mergeCell ref="F54:L54"/>
+    <mergeCell ref="M54:P54"/>
+    <mergeCell ref="D56:H56"/>
+    <mergeCell ref="I56:P56"/>
   </mergeCells>
   <conditionalFormatting sqref="B7:B42">
     <cfRule type="duplicateValues" dxfId="2" priority="1" stopIfTrue="1"/>

</xml_diff>